<commit_message>
feat: upgrade wishlist sheet to dual authentic web scenery/facility images and 8 columns
</commit_message>
<xml_diff>
--- a/曼谷自由行心願清單.xlsx
+++ b/曼谷自由行心願清單.xlsx
@@ -208,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -272,6 +272,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -372,9 +378,31 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -389,20 +417,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -417,20 +467,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -445,20 +517,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -473,20 +567,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -501,20 +617,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -529,20 +667,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -557,20 +717,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -585,20 +767,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -613,20 +817,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -641,20 +867,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -669,20 +917,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -697,20 +967,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -725,20 +1017,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -753,20 +1067,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -781,20 +1117,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -809,20 +1167,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -837,20 +1217,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -865,20 +1267,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -893,20 +1317,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -921,20 +1367,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -949,20 +1417,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -977,20 +1467,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1005,20 +1517,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1033,20 +1567,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1061,20 +1617,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1089,20 +1667,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1117,20 +1717,42 @@
     <ext cx="1047750" cy="685800"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1161,6 +1783,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1186,6 +1811,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1211,6 +1839,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1236,6 +1867,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1261,6 +1895,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1286,6 +1923,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1311,6 +1951,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1336,6 +1979,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1361,6 +2007,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1386,6 +2035,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1411,6 +2063,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1436,6 +2091,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1461,6 +2119,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1486,6 +2147,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1511,6 +2175,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1536,6 +2203,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1561,6 +2231,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1586,6 +2259,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1611,6 +2287,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1636,6 +2315,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1661,6 +2343,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1686,6 +2371,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1711,6 +2399,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1736,6 +2427,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1761,6 +2455,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1786,6 +2483,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1811,6 +2511,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1836,6 +2539,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1861,6 +2567,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1886,6 +2595,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1911,6 +2623,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1936,6 +2651,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1961,6 +2679,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1986,6 +2707,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2011,6 +2735,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2036,6 +2763,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2061,6 +2791,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2086,6 +2819,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2111,6 +2847,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2136,6 +2875,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2161,6 +2903,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2186,6 +2931,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2211,6 +2959,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2236,6 +2987,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2261,6 +3015,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2286,6 +3043,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2311,6 +3071,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2336,6 +3099,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2361,6 +3127,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2386,6 +3155,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2411,6 +3183,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2436,6 +3211,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2461,6 +3239,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2486,6 +3267,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2511,6 +3295,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2536,6 +3323,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2561,6 +3351,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2586,6 +3379,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2611,6 +3407,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2636,6 +3435,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2661,6 +3463,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2686,6 +3491,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2711,6 +3519,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2736,6 +3547,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2761,6 +3575,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2786,6 +3603,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2811,6 +3631,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2836,6 +3659,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2861,6 +3687,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2886,6 +3715,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2911,6 +3743,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2936,6 +3771,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2961,6 +3799,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2986,6 +3827,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3011,6 +3855,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3036,6 +3883,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3061,6 +3911,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3086,6 +3939,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3111,6 +3967,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3136,6 +3995,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3161,6 +4023,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3186,6 +4051,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3211,6 +4079,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3236,6 +4107,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3261,6 +4135,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3286,6 +4163,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3311,6 +4191,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3336,6 +4219,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3361,6 +4247,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3386,6 +4275,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3411,6 +4303,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3436,6 +4331,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3461,6 +4359,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3486,6 +4387,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3511,6 +4415,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3536,6 +4443,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3561,6 +4471,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3586,6 +4499,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3611,6 +4527,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3636,6 +4555,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3661,6 +4583,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3686,6 +4611,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3711,6 +4639,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3736,6 +4667,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3761,6 +4695,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3786,6 +4723,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3811,6 +4751,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3836,6 +4779,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3861,6 +4807,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3886,6 +4835,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3911,6 +4863,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3936,6 +4891,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3961,6 +4919,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3986,6 +4947,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4011,6 +4975,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4036,6 +5003,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4061,6 +5031,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4086,6 +5059,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4111,6 +5087,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4136,6 +5115,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4161,6 +5143,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4186,6 +5171,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4211,6 +5199,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4236,6 +5227,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4261,6 +5255,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4286,6 +5283,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4311,6 +5311,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4336,6 +5339,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4361,6 +5367,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4386,6 +5395,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4411,6 +5423,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4436,6 +5451,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4461,6 +5479,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4486,6 +5507,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4511,6 +5535,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4536,6 +5563,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4561,6 +5591,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4586,6 +5619,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4611,6 +5647,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4636,6 +5675,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4661,6 +5703,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4686,6 +5731,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4711,6 +5759,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4736,6 +5787,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4761,6 +5815,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4786,6 +5843,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4811,6 +5871,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4836,6 +5899,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4861,6 +5927,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4886,6 +5955,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4911,6 +5983,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4936,6 +6011,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4961,6 +6039,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4986,6 +6067,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5011,6 +6095,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5036,6 +6123,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5061,6 +6151,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5086,6 +6179,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5111,6 +6207,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5136,6 +6235,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5161,6 +6263,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5186,6 +6291,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5211,6 +6319,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5236,6 +6347,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5261,6 +6375,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5286,6 +6403,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5311,6 +6431,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5336,6 +6459,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5361,6 +6487,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5386,6 +6515,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5411,6 +6543,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5436,6 +6571,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5461,6 +6599,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5486,6 +6627,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5511,6 +6655,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5536,6 +6683,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5561,6 +6711,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5586,6 +6739,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5611,6 +6767,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5636,6 +6795,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5661,6 +6823,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5686,6 +6851,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5711,6 +6879,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5736,6 +6907,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5761,6 +6935,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5786,6 +6963,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5811,6 +6991,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5836,6 +7019,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5861,6 +7047,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5886,6 +7075,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5911,6 +7103,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5936,6 +7131,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5961,6 +7159,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -5986,6 +7187,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6011,6 +7215,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6036,6 +7243,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6061,6 +7271,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6086,6 +7299,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6111,6 +7327,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6136,6 +7355,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6161,6 +7383,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6186,6 +7411,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6211,6 +7439,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6236,6 +7467,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6261,6 +7495,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6286,6 +7523,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6311,6 +7551,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6336,6 +7579,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6361,6 +7607,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6386,6 +7635,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6411,6 +7663,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6436,6 +7691,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6461,6 +7719,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6486,6 +7747,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6511,6 +7775,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6536,6 +7803,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6561,6 +7831,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6586,6 +7859,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6611,6 +7887,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6636,6 +7915,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6932,7 +8214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6941,7 +8223,8 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -6950,6 +8233,7 @@
           <t>🇹🇭 曼谷自由行心願清單</t>
         </is>
       </c>
+      <c r="H1" s="10" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -6982,9 +8266,14 @@
           <t>備註</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>圖片</t>
+      <c r="G2" s="24" t="inlineStr">
+        <is>
+          <t>圖片 1 (環境/外觀/風景)</t>
+        </is>
+      </c>
+      <c r="H2" s="24" t="inlineStr">
+        <is>
+          <t>圖片 2 (特色/餐點/設施)</t>
         </is>
       </c>
     </row>
@@ -7020,6 +8309,7 @@
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr"/>
+      <c r="H3" s="25" t="n"/>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -7053,6 +8343,7 @@
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
+      <c r="H4" s="25" t="n"/>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -7086,6 +8377,7 @@
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr"/>
+      <c r="H5" s="25" t="n"/>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -7119,6 +8411,7 @@
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="25" t="n"/>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -7152,6 +8445,7 @@
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="25" t="n"/>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -7185,6 +8479,7 @@
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="25" t="n"/>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -7218,6 +8513,7 @@
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="25" t="n"/>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -7251,6 +8547,7 @@
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr"/>
+      <c r="H10" s="25" t="n"/>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -7284,6 +8581,7 @@
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="25" t="n"/>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -7317,6 +8615,7 @@
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr"/>
+      <c r="H12" s="25" t="n"/>
     </row>
     <row r="13" ht="70" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -7350,6 +8649,7 @@
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="25" t="n"/>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -7383,6 +8683,7 @@
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr"/>
+      <c r="H14" s="25" t="n"/>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -7416,6 +8717,7 @@
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="25" t="n"/>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -7449,6 +8751,7 @@
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr"/>
+      <c r="H16" s="25" t="n"/>
     </row>
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -7482,6 +8785,7 @@
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="25" t="n"/>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -7515,6 +8819,7 @@
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="25" t="n"/>
     </row>
     <row r="19" ht="70" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -7548,6 +8853,7 @@
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="25" t="n"/>
     </row>
     <row r="20" ht="70" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -7581,6 +8887,7 @@
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="25" t="n"/>
     </row>
     <row r="21" ht="70" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -7614,6 +8921,7 @@
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="25" t="n"/>
     </row>
     <row r="22" ht="70" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -7647,6 +8955,7 @@
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="25" t="n"/>
     </row>
     <row r="23" ht="70" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -7680,6 +8989,7 @@
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr"/>
+      <c r="H23" s="25" t="n"/>
     </row>
     <row r="24" ht="70" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -7713,6 +9023,7 @@
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr"/>
+      <c r="H24" s="25" t="n"/>
     </row>
     <row r="25" ht="70" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -7746,6 +9057,7 @@
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr"/>
+      <c r="H25" s="25" t="n"/>
     </row>
     <row r="26" ht="70" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -7779,6 +9091,7 @@
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="25" t="n"/>
     </row>
     <row r="27" ht="70" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -7812,6 +9125,7 @@
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr"/>
+      <c r="H27" s="25" t="n"/>
     </row>
     <row r="28" ht="70" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -7845,6 +9159,7 @@
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="25" t="n"/>
     </row>
     <row r="29" ht="70" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -7878,6 +9193,7 @@
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr"/>
+      <c r="H29" s="25" t="n"/>
     </row>
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -7911,10 +9227,11 @@
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr"/>
+      <c r="H30" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
@@ -8527,15 +9844,15 @@
           <t>🇹🇭 曼谷自由行 影音參考影片提及地點全攻略 (含米其林指南推薦專區)</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
-      <c r="D1" s="10" t="n"/>
-      <c r="E1" s="10" t="n"/>
-      <c r="F1" s="10" t="n"/>
-      <c r="G1" s="10" t="n"/>
-      <c r="H1" s="10" t="n"/>
-      <c r="I1" s="10" t="n"/>
-      <c r="J1" s="10" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="14" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
@@ -8543,15 +9860,15 @@
           <t>🏆 【精選專區】影音推薦「米其林指南」必吃美食清單（13處必比登推薦與星級入選）</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="n"/>
-      <c r="H2" s="10" t="n"/>
-      <c r="I2" s="10" t="n"/>
-      <c r="J2" s="10" t="n"/>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="13" t="n"/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="13" t="n"/>
+      <c r="J2" s="14" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
@@ -9235,15 +10552,15 @@
           <t>🎬 【完整收錄】8 部 YouTube 攻略影片逐項地點與精確時間軸總覽（美食 / 景點 / 住宿 / 購物）</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="10" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="14" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="17" t="inlineStr">

</xml_diff>